<commit_message>
help notes, baccarat cards, login fix
</commit_message>
<xml_diff>
--- a/db_storage/knowledge_base.xlsx
+++ b/db_storage/knowledge_base.xlsx
@@ -6,6 +6,8 @@
     <sheet name="__meta__" sheetId="1" r:id="rId1"/>
     <sheet name="__schema__" sheetId="2" r:id="rId2"/>
     <sheet name="articles" sheetId="3" r:id="rId3"/>
+    <sheet name="help_notes" sheetId="4" r:id="rId4"/>
+    <sheet name="qna" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -420,7 +422,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -438,9 +440,25 @@
         <v>id,title,category,status,publisher,created_at,updated_at</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>help_notes</v>
+      </c>
+      <c r="B3" t="str">
+        <v>id,notes,priority,created_at,updated_at</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>qna</v>
+      </c>
+      <c r="B4" t="str">
+        <v>id,question,answer,options,priority,created_at,updated_at</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -509,4 +527,174 @@
     <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>notes</v>
+      </c>
+      <c r="C1" t="str">
+        <v>priority</v>
+      </c>
+      <c r="D1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="E1" t="str">
+        <v>updated_at</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>For BT Operator there are no Slots log</v>
+      </c>
+      <c r="C2" t="str">
+        <v>1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-04-25T17:22:11.332Z</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-04-26T06:56:23.890Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Authenticate creates a secure session token before game launch.</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-04-26T06:59:35.440Z</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-04-26T07:11:00.048Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="str">
+        <v>GetCasinoGames returns available games for lobby building</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-04-26T06:59:56.404Z</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-04-26T06:59:56.404Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Crash games report results in a single structured sm_result string</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-04-26T07:00:20.243Z</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-04-26T07:00:20.243Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="str">
+        <v>sm_result includes bet, multiplier, final multiplier, and win/loss status</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-04-26T07:00:34.002Z</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-04-26T07:00:34.002Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>question</v>
+      </c>
+      <c r="C1" t="str">
+        <v>answer</v>
+      </c>
+      <c r="D1" t="str">
+        <v>options</v>
+      </c>
+      <c r="E1" t="str">
+        <v>priority</v>
+      </c>
+      <c r="F1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="G1" t="str">
+        <v>updated_at</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>3</v>
+      </c>
+      <c r="B2" t="str">
+        <v>What is fd</v>
+      </c>
+      <c r="C2" t="str">
+        <v>sdfdf</v>
+      </c>
+      <c r="D2" t="str">
+        <v>ds,sdfdf</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-04-26T06:07:30.441Z</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-04-26T09:13:36.799Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
qna and other crash games result and other
</commit_message>
<xml_diff>
--- a/db_storage/knowledge_base.xlsx
+++ b/db_storage/knowledge_base.xlsx
@@ -644,7 +644,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -674,13 +674,13 @@
         <v>3</v>
       </c>
       <c r="B2" t="str">
-        <v>What is fd</v>
+        <v>For the BT operator, which URL is used to launch the game?</v>
       </c>
       <c r="C2" t="str">
-        <v>sdfdf</v>
+        <v>opengame.do</v>
       </c>
       <c r="D2" t="str">
-        <v>ds,sdfdf</v>
+        <v>opengame.do,playgame.do</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -689,12 +689,58 @@
         <v>2026-04-26T06:07:30.441Z</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-26T09:13:36.799Z</v>
+        <v>2026-05-03T09:16:12.001Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>4</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Do we get the SLOTS log for the BT operator?</v>
+      </c>
+      <c r="C3" t="str">
+        <v>No</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Yes,No</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-05-03T09:16:58.301Z</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-05-03T09:16:58.301Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>5</v>
+      </c>
+      <c r="B4" t="str">
+        <v>How to know if the game is enabled for FreeChips?</v>
+      </c>
+      <c r="C4" t="str">
+        <v>In GetCasinoGames Check for fcAvailable param</v>
+      </c>
+      <c r="D4" t="str">
+        <v>In GetCasinoGames Check for fcAvailable param,Check in the Database,Under Casino Details in Table Config</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-05-03T09:22:32.503Z</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-05-03T09:22:32.503Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: update favicon and knowledge base files, remove unused SVG assets
</commit_message>
<xml_diff>
--- a/db_storage/knowledge_base.xlsx
+++ b/db_storage/knowledge_base.xlsx
@@ -531,7 +531,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -550,94 +550,9 @@
         <v>updated_at</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>For BT Operator there are no Slots log</v>
-      </c>
-      <c r="C2" t="str">
-        <v>1</v>
-      </c>
-      <c r="D2" t="str">
-        <v>2026-04-25T17:22:11.332Z</v>
-      </c>
-      <c r="E2" t="str">
-        <v>2026-04-26T06:56:23.890Z</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>3</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Authenticate creates a secure session token before game launch.</v>
-      </c>
-      <c r="C3">
-        <v>3</v>
-      </c>
-      <c r="D3" t="str">
-        <v>2026-04-26T06:59:35.440Z</v>
-      </c>
-      <c r="E3" t="str">
-        <v>2026-04-27T05:09:23.681Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" t="str">
-        <v>GetCasinoGames returns available games for lobby building</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="str">
-        <v>2026-04-26T06:59:56.404Z</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2026-04-26T06:59:56.404Z</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>5</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Crash games report results in a single structured sm_result string</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="str">
-        <v>2026-04-26T07:00:20.243Z</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2026-04-26T07:00:20.243Z</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>6</v>
-      </c>
-      <c r="B6" t="str">
-        <v>sm_result includes bet, multiplier, final multiplier, and win/loss status</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6" t="str">
-        <v>2026-04-26T07:00:34.002Z</v>
-      </c>
-      <c r="E6" t="str">
-        <v>2026-04-26T07:00:34.002Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(bet-history): enhance BetHistoryForm with date presets and time range shifting functionality
feat(log-exp): improve IntegratedDateTimeRangePicker layout and interaction

feat(round-details): implement bulk ID input limit and validation in MultiRoundDetailsForm

feat(round-details): add keyboard navigation for MultiRoundTabs and improve tab loading indicators

fix(round-audit): optimize log retrieval and ID assignment in useLogState and useIsolatedLogs hooks

fix(round-audit): enhance prefetching logic for transaction logs with retry mechanism

feat(excel-engine): refine findFeatureList function to accept roles array for filtering

feat(bet-history): create DatePresetDropdown for quick date selection in BetHistoryForm
</commit_message>
<xml_diff>
--- a/db_storage/knowledge_base.xlsx
+++ b/db_storage/knowledge_base.xlsx
@@ -531,7 +531,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -550,9 +550,94 @@
         <v>updated_at</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>For BT Operator there are no Slots log</v>
+      </c>
+      <c r="C2" t="str">
+        <v>1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-04-25T17:22:11.332Z</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-04-26T06:56:23.890Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Authenticate creates a secure session token before game launch.</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-04-26T06:59:35.440Z</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-04-27T05:09:23.681Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="str">
+        <v>GetCasinoGames returns available games for lobby building</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-04-26T06:59:56.404Z</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-04-26T06:59:56.404Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Crash games report results in a single structured sm_result string</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-04-26T07:00:20.243Z</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-04-26T07:00:20.243Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="str">
+        <v>sm_result includes bet, multiplier, final multiplier, and win/loss status</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-04-26T07:00:34.002Z</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-04-26T07:00:34.002Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>